<commit_message>
feat: initialize OBE curriculum documentation, analysis matrices, assessment rubrics, and supporting conversion scripts for SISTEKIN 2026.
</commit_message>
<xml_diff>
--- a/KURIKULUM2026_REVISI/003_STANDAR_14_CPL_DAN_PEMETAAN_BoK_APTIKOM.xlsx
+++ b/KURIKULUM2026_REVISI/003_STANDAR_14_CPL_DAN_PEMETAAN_BoK_APTIKOM.xlsx
@@ -551,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P96"/>
+  <dimension ref="A1:P99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="69" customWidth="1" min="1" max="1"/>
@@ -1440,7 +1440,7 @@
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>4. MATRIKS SILANG CPL ↔ 19 BAHAN KAJIAN (BoK) IS2020 (APTIKOM v2.0)</t>
+          <t>4. MATRIKS SILANG CPL ↔ 21 BAHAN KAJIAN (BoK) IS2020 (APTIKOM v2.0)</t>
         </is>
       </c>
       <c r="B46" s="4" t="n"/>
@@ -2223,184 +2223,204 @@
       <c r="O66" s="8" t="inlineStr"/>
       <c r="P66" s="8" t="inlineStr"/>
     </row>
-    <row r="67"/>
-    <row r="68" ht="20" customHeight="1">
-      <c r="A68" s="3" t="inlineStr">
-        <is>
-          <t>5. MATRIKS SILANG CPL ↔ 14 BAHAN KAJIAN UTAMA (BoK) IT2017 (APTIKOM)</t>
-        </is>
-      </c>
-      <c r="B68" s="4" t="n"/>
-      <c r="C68" s="4" t="n"/>
-      <c r="D68" s="4" t="n"/>
-      <c r="E68" s="4" t="n"/>
-      <c r="F68" s="4" t="n"/>
-      <c r="G68" s="4" t="n"/>
-      <c r="H68" s="4" t="n"/>
-      <c r="I68" s="4" t="n"/>
-      <c r="J68" s="4" t="n"/>
-      <c r="K68" s="4" t="n"/>
-      <c r="L68" s="4" t="n"/>
-      <c r="M68" s="4" t="n"/>
-      <c r="N68" s="4" t="n"/>
-      <c r="O68" s="4" t="n"/>
-      <c r="P68" s="5" t="n"/>
-    </row>
-    <row r="69" ht="26" customHeight="1">
-      <c r="A69" s="6" t="inlineStr">
+    <row r="67" ht="16" customHeight="1">
+      <c r="A67" s="10" t="inlineStr">
+        <is>
+          <t>**BK-IS20**</t>
+        </is>
+      </c>
+      <c r="B67" s="10" t="inlineStr">
+        <is>
+          <t>*Ethics, Use and Implications for Society*</t>
+        </is>
+      </c>
+      <c r="C67" s="9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D67" s="9" t="inlineStr"/>
+      <c r="E67" s="10" t="inlineStr"/>
+      <c r="F67" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G67" s="10" t="inlineStr"/>
+      <c r="H67" s="10" t="inlineStr"/>
+      <c r="I67" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J67" s="10" t="inlineStr"/>
+      <c r="K67" s="10" t="inlineStr"/>
+      <c r="L67" s="10" t="inlineStr"/>
+      <c r="M67" s="10" t="inlineStr"/>
+      <c r="N67" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="O67" s="10" t="inlineStr"/>
+      <c r="P67" s="10" t="inlineStr"/>
+    </row>
+    <row r="68" ht="16" customHeight="1">
+      <c r="A68" s="8" t="inlineStr">
+        <is>
+          <t>**BK-IS21**</t>
+        </is>
+      </c>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>*Internship and Professional Practice*</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F68" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G68" s="8" t="inlineStr"/>
+      <c r="H68" s="8" t="inlineStr"/>
+      <c r="I68" s="8" t="inlineStr"/>
+      <c r="J68" s="8" t="inlineStr"/>
+      <c r="K68" s="8" t="inlineStr"/>
+      <c r="L68" s="8" t="inlineStr"/>
+      <c r="M68" s="8" t="inlineStr"/>
+      <c r="N68" s="8" t="inlineStr"/>
+      <c r="O68" s="8" t="inlineStr"/>
+      <c r="P68" s="8" t="inlineStr"/>
+    </row>
+    <row r="69"/>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>5. MATRIKS SILANG CPL ↔ 15 BAHAN KAJIAN UTAMA (BoK) IT2017 (APTIKOM)</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="n"/>
+      <c r="C70" s="4" t="n"/>
+      <c r="D70" s="4" t="n"/>
+      <c r="E70" s="4" t="n"/>
+      <c r="F70" s="4" t="n"/>
+      <c r="G70" s="4" t="n"/>
+      <c r="H70" s="4" t="n"/>
+      <c r="I70" s="4" t="n"/>
+      <c r="J70" s="4" t="n"/>
+      <c r="K70" s="4" t="n"/>
+      <c r="L70" s="4" t="n"/>
+      <c r="M70" s="4" t="n"/>
+      <c r="N70" s="4" t="n"/>
+      <c r="O70" s="4" t="n"/>
+      <c r="P70" s="5" t="n"/>
+    </row>
+    <row r="71" ht="26" customHeight="1">
+      <c r="A71" s="6" t="inlineStr">
         <is>
           <t>Kode Bahan Kajian (BoK)</t>
         </is>
       </c>
-      <c r="B69" s="6" t="inlineStr">
+      <c r="B71" s="6" t="inlineStr">
         <is>
           <t>Nomenklatur Bahan Kajian Utama IT2017</t>
         </is>
       </c>
-      <c r="C69" s="6" t="inlineStr">
+      <c r="C71" s="6" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="D69" s="6" t="inlineStr">
+      <c r="D71" s="6" t="inlineStr">
         <is>
           <t>KU1</t>
         </is>
       </c>
-      <c r="E69" s="6" t="inlineStr">
+      <c r="E71" s="6" t="inlineStr">
         <is>
           <t>KU2</t>
         </is>
       </c>
-      <c r="F69" s="6" t="inlineStr">
+      <c r="F71" s="6" t="inlineStr">
         <is>
           <t>KU3</t>
         </is>
       </c>
-      <c r="G69" s="6" t="inlineStr">
+      <c r="G71" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="H69" s="6" t="inlineStr">
+      <c r="H71" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="I69" s="6" t="inlineStr">
+      <c r="I71" s="6" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="J69" s="6" t="inlineStr">
+      <c r="J71" s="6" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="K69" s="6" t="inlineStr">
+      <c r="K71" s="6" t="inlineStr">
         <is>
           <t>KK1</t>
         </is>
       </c>
-      <c r="L69" s="6" t="inlineStr">
+      <c r="L71" s="6" t="inlineStr">
         <is>
           <t>KK2</t>
         </is>
       </c>
-      <c r="M69" s="6" t="inlineStr">
+      <c r="M71" s="6" t="inlineStr">
         <is>
           <t>KK3</t>
         </is>
       </c>
-      <c r="N69" s="6" t="inlineStr">
+      <c r="N71" s="6" t="inlineStr">
         <is>
           <t>KK4</t>
         </is>
       </c>
-      <c r="O69" s="6" t="inlineStr">
+      <c r="O71" s="6" t="inlineStr">
         <is>
           <t>KK5</t>
         </is>
       </c>
-      <c r="P69" s="6" t="inlineStr">
+      <c r="P71" s="6" t="inlineStr">
         <is>
           <t>KK6</t>
         </is>
       </c>
-    </row>
-    <row r="70" ht="16" customHeight="1">
-      <c r="A70" s="8" t="inlineStr">
-        <is>
-          <t>**BK-IT01**</t>
-        </is>
-      </c>
-      <c r="B70" s="8" t="inlineStr">
-        <is>
-          <t>*Information Technology Fundamentals*</t>
-        </is>
-      </c>
-      <c r="C70" s="7" t="inlineStr"/>
-      <c r="D70" s="7" t="inlineStr"/>
-      <c r="E70" s="8" t="inlineStr"/>
-      <c r="F70" s="8" t="inlineStr"/>
-      <c r="G70" s="8" t="inlineStr"/>
-      <c r="H70" s="8" t="inlineStr"/>
-      <c r="I70" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J70" s="8" t="inlineStr"/>
-      <c r="K70" s="8" t="inlineStr"/>
-      <c r="L70" s="8" t="inlineStr"/>
-      <c r="M70" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N70" s="8" t="inlineStr"/>
-      <c r="O70" s="8" t="inlineStr"/>
-      <c r="P70" s="8" t="inlineStr"/>
-    </row>
-    <row r="71" ht="16" customHeight="1">
-      <c r="A71" s="10" t="inlineStr">
-        <is>
-          <t>**BK-IT02**</t>
-        </is>
-      </c>
-      <c r="B71" s="10" t="inlineStr">
-        <is>
-          <t>*Applied AI &amp; Intelligent Technologies*</t>
-        </is>
-      </c>
-      <c r="C71" s="9" t="inlineStr"/>
-      <c r="D71" s="9" t="inlineStr"/>
-      <c r="E71" s="10" t="inlineStr"/>
-      <c r="F71" s="10" t="inlineStr"/>
-      <c r="G71" s="10" t="inlineStr"/>
-      <c r="H71" s="10" t="inlineStr"/>
-      <c r="I71" s="10" t="inlineStr"/>
-      <c r="J71" s="10" t="inlineStr"/>
-      <c r="K71" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L71" s="10" t="inlineStr"/>
-      <c r="M71" s="10" t="inlineStr"/>
-      <c r="N71" s="10" t="inlineStr"/>
-      <c r="O71" s="10" t="inlineStr"/>
-      <c r="P71" s="10" t="inlineStr"/>
     </row>
     <row r="72" ht="16" customHeight="1">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>**BK-IT03**</t>
+          <t>**BK-IT01**</t>
         </is>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>*Networking &amp; Communications*</t>
+          <t>*Information Technology Fundamentals*</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr"/>
@@ -2429,12 +2449,12 @@
     <row r="73" ht="16" customHeight="1">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>**BK-IT04**</t>
+          <t>**BK-IT02**</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>*Platform Technologies &amp; Web/Mobile*</t>
+          <t>*Applied AI &amp; Intelligent Technologies*</t>
         </is>
       </c>
       <c r="C73" s="9" t="inlineStr"/>
@@ -2444,31 +2464,27 @@
       <c r="G73" s="10" t="inlineStr"/>
       <c r="H73" s="10" t="inlineStr"/>
       <c r="I73" s="10" t="inlineStr"/>
-      <c r="J73" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K73" s="10" t="inlineStr"/>
+      <c r="J73" s="10" t="inlineStr"/>
+      <c r="K73" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L73" s="10" t="inlineStr"/>
       <c r="M73" s="10" t="inlineStr"/>
       <c r="N73" s="10" t="inlineStr"/>
-      <c r="O73" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="O73" s="10" t="inlineStr"/>
       <c r="P73" s="10" t="inlineStr"/>
     </row>
     <row r="74" ht="16" customHeight="1">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t>**BK-IT05**</t>
+          <t>**BK-IT03**</t>
         </is>
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>*Cloud Computing &amp; Virtualization*</t>
+          <t>*Networking &amp; Communications*</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr"/>
@@ -2497,12 +2513,12 @@
     <row r="75" ht="16" customHeight="1">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>**BK-IT06**</t>
+          <t>**BK-IT04**</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>*Cybersecurity Principles &amp; Defense*</t>
+          <t>*Platform Technologies &amp; Web/Mobile*</t>
         </is>
       </c>
       <c r="C75" s="9" t="inlineStr"/>
@@ -2511,36 +2527,32 @@
       <c r="F75" s="10" t="inlineStr"/>
       <c r="G75" s="10" t="inlineStr"/>
       <c r="H75" s="10" t="inlineStr"/>
-      <c r="I75" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J75" s="10" t="inlineStr"/>
+      <c r="I75" s="10" t="inlineStr"/>
+      <c r="J75" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K75" s="10" t="inlineStr"/>
       <c r="L75" s="10" t="inlineStr"/>
-      <c r="M75" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N75" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="O75" s="10" t="inlineStr"/>
+      <c r="M75" s="10" t="inlineStr"/>
+      <c r="N75" s="10" t="inlineStr"/>
+      <c r="O75" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="P75" s="10" t="inlineStr"/>
     </row>
     <row r="76" ht="16" customHeight="1">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>**BK-IT07**</t>
+          <t>**BK-IT05**</t>
         </is>
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>*System Integration and Architecture*</t>
+          <t>*Cloud Computing &amp; Virtualization*</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr"/>
@@ -2563,22 +2575,18 @@
         </is>
       </c>
       <c r="N76" s="8" t="inlineStr"/>
-      <c r="O76" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="O76" s="8" t="inlineStr"/>
       <c r="P76" s="8" t="inlineStr"/>
     </row>
     <row r="77" ht="16" customHeight="1">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>**BK-IT08**</t>
+          <t>**BK-IT06**</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>*IT Service Management &amp; Governance*</t>
+          <t>*Cybersecurity Principles &amp; Defense*</t>
         </is>
       </c>
       <c r="C77" s="9" t="inlineStr"/>
@@ -2595,7 +2603,11 @@
       <c r="J77" s="10" t="inlineStr"/>
       <c r="K77" s="10" t="inlineStr"/>
       <c r="L77" s="10" t="inlineStr"/>
-      <c r="M77" s="10" t="inlineStr"/>
+      <c r="M77" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N77" s="10" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2607,12 +2619,12 @@
     <row r="78" ht="16" customHeight="1">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>**BK-IT09**</t>
+          <t>**BK-IT07**</t>
         </is>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>*Data Analytics &amp; Information Visualization*</t>
+          <t>*System Integration and Architecture*</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr"/>
@@ -2621,32 +2633,36 @@
       <c r="F78" s="8" t="inlineStr"/>
       <c r="G78" s="8" t="inlineStr"/>
       <c r="H78" s="8" t="inlineStr"/>
-      <c r="I78" s="8" t="inlineStr"/>
-      <c r="J78" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I78" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J78" s="8" t="inlineStr"/>
       <c r="K78" s="8" t="inlineStr"/>
-      <c r="L78" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M78" s="8" t="inlineStr"/>
+      <c r="L78" s="8" t="inlineStr"/>
+      <c r="M78" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N78" s="8" t="inlineStr"/>
-      <c r="O78" s="8" t="inlineStr"/>
+      <c r="O78" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="P78" s="8" t="inlineStr"/>
     </row>
     <row r="79" ht="16" customHeight="1">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>**BK-IT10**</t>
+          <t>**BK-IT08**</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t>*User Experience &amp; Interaction Design*</t>
+          <t>*IT Service Management &amp; Governance*</t>
         </is>
       </c>
       <c r="C79" s="9" t="inlineStr"/>
@@ -2655,32 +2671,32 @@
       <c r="F79" s="10" t="inlineStr"/>
       <c r="G79" s="10" t="inlineStr"/>
       <c r="H79" s="10" t="inlineStr"/>
-      <c r="I79" s="10" t="inlineStr"/>
-      <c r="J79" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I79" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J79" s="10" t="inlineStr"/>
       <c r="K79" s="10" t="inlineStr"/>
       <c r="L79" s="10" t="inlineStr"/>
       <c r="M79" s="10" t="inlineStr"/>
-      <c r="N79" s="10" t="inlineStr"/>
-      <c r="O79" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="N79" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="O79" s="10" t="inlineStr"/>
       <c r="P79" s="10" t="inlineStr"/>
     </row>
     <row r="80" ht="16" customHeight="1">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>**BK-IT11**</t>
+          <t>**BK-IT09**</t>
         </is>
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>*Software Development Practices*</t>
+          <t>*Data Analytics &amp; Information Visualization*</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr"/>
@@ -2696,25 +2712,25 @@
         </is>
       </c>
       <c r="K80" s="8" t="inlineStr"/>
-      <c r="L80" s="8" t="inlineStr"/>
+      <c r="L80" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M80" s="8" t="inlineStr"/>
       <c r="N80" s="8" t="inlineStr"/>
-      <c r="O80" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="O80" s="8" t="inlineStr"/>
       <c r="P80" s="8" t="inlineStr"/>
     </row>
     <row r="81" ht="16" customHeight="1">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>**BK-IT12**</t>
+          <t>**BK-IT10**</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>*IT Risk Management and Compliance*</t>
+          <t>*User Experience &amp; Interaction Design*</t>
         </is>
       </c>
       <c r="C81" s="9" t="inlineStr"/>
@@ -2724,27 +2740,31 @@
       <c r="G81" s="10" t="inlineStr"/>
       <c r="H81" s="10" t="inlineStr"/>
       <c r="I81" s="10" t="inlineStr"/>
-      <c r="J81" s="10" t="inlineStr"/>
+      <c r="J81" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K81" s="10" t="inlineStr"/>
       <c r="L81" s="10" t="inlineStr"/>
       <c r="M81" s="10" t="inlineStr"/>
-      <c r="N81" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="O81" s="10" t="inlineStr"/>
+      <c r="N81" s="10" t="inlineStr"/>
+      <c r="O81" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="P81" s="10" t="inlineStr"/>
     </row>
     <row r="82" ht="16" customHeight="1">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t>**BK-IT13**</t>
+          <t>**BK-IT11**</t>
         </is>
       </c>
       <c r="B82" s="8" t="inlineStr">
         <is>
-          <t>*Technology Entrepreneurship*</t>
+          <t>*Software Development Practices*</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr"/>
@@ -2754,27 +2774,31 @@
       <c r="G82" s="8" t="inlineStr"/>
       <c r="H82" s="8" t="inlineStr"/>
       <c r="I82" s="8" t="inlineStr"/>
-      <c r="J82" s="8" t="inlineStr"/>
+      <c r="J82" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K82" s="8" t="inlineStr"/>
       <c r="L82" s="8" t="inlineStr"/>
       <c r="M82" s="8" t="inlineStr"/>
       <c r="N82" s="8" t="inlineStr"/>
-      <c r="O82" s="8" t="inlineStr"/>
-      <c r="P82" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="O82" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="P82" s="8" t="inlineStr"/>
     </row>
     <row r="83" ht="16" customHeight="1">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>**BK-IT14**</t>
+          <t>**BK-IT12**</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>*IoT and Embedded Smart Systems*</t>
+          <t>*IT Risk Management and Compliance*</t>
         </is>
       </c>
       <c r="C83" s="9" t="inlineStr"/>
@@ -2785,490 +2809,592 @@
       <c r="H83" s="10" t="inlineStr"/>
       <c r="I83" s="10" t="inlineStr"/>
       <c r="J83" s="10" t="inlineStr"/>
-      <c r="K83" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K83" s="10" t="inlineStr"/>
       <c r="L83" s="10" t="inlineStr"/>
-      <c r="M83" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N83" s="10" t="inlineStr"/>
+      <c r="M83" s="10" t="inlineStr"/>
+      <c r="N83" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="O83" s="10" t="inlineStr"/>
       <c r="P83" s="10" t="inlineStr"/>
     </row>
-    <row r="84"/>
-    <row r="85" ht="20" customHeight="1">
-      <c r="A85" s="3" t="inlineStr">
+    <row r="84" ht="16" customHeight="1">
+      <c r="A84" s="8" t="inlineStr">
+        <is>
+          <t>**BK-IT13**</t>
+        </is>
+      </c>
+      <c r="B84" s="8" t="inlineStr">
+        <is>
+          <t>*Technology Entrepreneurship*</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr"/>
+      <c r="D84" s="7" t="inlineStr"/>
+      <c r="E84" s="8" t="inlineStr"/>
+      <c r="F84" s="8" t="inlineStr"/>
+      <c r="G84" s="8" t="inlineStr"/>
+      <c r="H84" s="8" t="inlineStr"/>
+      <c r="I84" s="8" t="inlineStr"/>
+      <c r="J84" s="8" t="inlineStr"/>
+      <c r="K84" s="8" t="inlineStr"/>
+      <c r="L84" s="8" t="inlineStr"/>
+      <c r="M84" s="8" t="inlineStr"/>
+      <c r="N84" s="8" t="inlineStr"/>
+      <c r="O84" s="8" t="inlineStr"/>
+      <c r="P84" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="16" customHeight="1">
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t>**BK-IT14**</t>
+        </is>
+      </c>
+      <c r="B85" s="10" t="inlineStr">
+        <is>
+          <t>*IoT and Embedded Smart Systems*</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="inlineStr"/>
+      <c r="D85" s="9" t="inlineStr"/>
+      <c r="E85" s="10" t="inlineStr"/>
+      <c r="F85" s="10" t="inlineStr"/>
+      <c r="G85" s="10" t="inlineStr"/>
+      <c r="H85" s="10" t="inlineStr"/>
+      <c r="I85" s="10" t="inlineStr"/>
+      <c r="J85" s="10" t="inlineStr"/>
+      <c r="K85" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L85" s="10" t="inlineStr"/>
+      <c r="M85" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N85" s="10" t="inlineStr"/>
+      <c r="O85" s="10" t="inlineStr"/>
+      <c r="P85" s="10" t="inlineStr"/>
+    </row>
+    <row r="86" ht="16" customHeight="1">
+      <c r="A86" s="8" t="inlineStr">
+        <is>
+          <t>**BK-IT15**</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>*Global Professional Practice*</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F86" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G86" s="8" t="inlineStr"/>
+      <c r="H86" s="8" t="inlineStr"/>
+      <c r="I86" s="8" t="inlineStr"/>
+      <c r="J86" s="8" t="inlineStr"/>
+      <c r="K86" s="8" t="inlineStr"/>
+      <c r="L86" s="8" t="inlineStr"/>
+      <c r="M86" s="8" t="inlineStr"/>
+      <c r="N86" s="8" t="inlineStr"/>
+      <c r="O86" s="8" t="inlineStr"/>
+      <c r="P86" s="8" t="inlineStr"/>
+    </row>
+    <row r="87"/>
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="3" t="inlineStr">
         <is>
           <t>6. MATRIKS PEMETAAN CPL ↔ 4 PROFIL LULUSAN (PL)</t>
         </is>
       </c>
-      <c r="B85" s="4" t="n"/>
-      <c r="C85" s="4" t="n"/>
-      <c r="D85" s="4" t="n"/>
-      <c r="E85" s="4" t="n"/>
-      <c r="F85" s="4" t="n"/>
-      <c r="G85" s="4" t="n"/>
-      <c r="H85" s="4" t="n"/>
-      <c r="I85" s="4" t="n"/>
-      <c r="J85" s="4" t="n"/>
-      <c r="K85" s="4" t="n"/>
-      <c r="L85" s="4" t="n"/>
-      <c r="M85" s="4" t="n"/>
-      <c r="N85" s="4" t="n"/>
-      <c r="O85" s="4" t="n"/>
-      <c r="P85" s="5" t="n"/>
-    </row>
-    <row r="86" ht="26" customHeight="1">
-      <c r="A86" s="6" t="inlineStr">
+      <c r="B88" s="4" t="n"/>
+      <c r="C88" s="4" t="n"/>
+      <c r="D88" s="4" t="n"/>
+      <c r="E88" s="4" t="n"/>
+      <c r="F88" s="4" t="n"/>
+      <c r="G88" s="4" t="n"/>
+      <c r="H88" s="4" t="n"/>
+      <c r="I88" s="4" t="n"/>
+      <c r="J88" s="4" t="n"/>
+      <c r="K88" s="4" t="n"/>
+      <c r="L88" s="4" t="n"/>
+      <c r="M88" s="4" t="n"/>
+      <c r="N88" s="4" t="n"/>
+      <c r="O88" s="4" t="n"/>
+      <c r="P88" s="5" t="n"/>
+    </row>
+    <row r="89" ht="26" customHeight="1">
+      <c r="A89" s="6" t="inlineStr">
         <is>
           <t>Profil Lulusan SISTEKIN 2026</t>
         </is>
       </c>
-      <c r="B86" s="6" t="inlineStr">
+      <c r="B89" s="6" t="inlineStr">
         <is>
           <t>Peminatan Terkait</t>
         </is>
       </c>
-      <c r="C86" s="6" t="inlineStr">
+      <c r="C89" s="6" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="D86" s="6" t="inlineStr">
+      <c r="D89" s="6" t="inlineStr">
         <is>
           <t>KU1</t>
         </is>
       </c>
-      <c r="E86" s="6" t="inlineStr">
+      <c r="E89" s="6" t="inlineStr">
         <is>
           <t>KU2</t>
         </is>
       </c>
-      <c r="F86" s="6" t="inlineStr">
+      <c r="F89" s="6" t="inlineStr">
         <is>
           <t>KU3</t>
         </is>
       </c>
-      <c r="G86" s="6" t="inlineStr">
+      <c r="G89" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="H86" s="6" t="inlineStr">
+      <c r="H89" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="I86" s="6" t="inlineStr">
+      <c r="I89" s="6" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="J86" s="6" t="inlineStr">
+      <c r="J89" s="6" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="K86" s="6" t="inlineStr">
+      <c r="K89" s="6" t="inlineStr">
         <is>
           <t>KK1</t>
         </is>
       </c>
-      <c r="L86" s="6" t="inlineStr">
+      <c r="L89" s="6" t="inlineStr">
         <is>
           <t>KK2</t>
         </is>
       </c>
-      <c r="M86" s="6" t="inlineStr">
+      <c r="M89" s="6" t="inlineStr">
         <is>
           <t>KK3</t>
         </is>
       </c>
-      <c r="N86" s="6" t="inlineStr">
+      <c r="N89" s="6" t="inlineStr">
         <is>
           <t>KK4</t>
         </is>
       </c>
-      <c r="O86" s="6" t="inlineStr">
+      <c r="O89" s="6" t="inlineStr">
         <is>
           <t>KK5</t>
         </is>
       </c>
-      <c r="P86" s="6" t="inlineStr">
+      <c r="P89" s="6" t="inlineStr">
         <is>
           <t>KK6</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="16" customHeight="1">
-      <c r="A87" s="8" t="inlineStr">
+    <row r="90" ht="16" customHeight="1">
+      <c r="A90" s="8" t="inlineStr">
         <is>
           <t>**PL-1: Intelligent IS Developer &amp; AI Engineer**</t>
         </is>
       </c>
-      <c r="B87" s="7" t="inlineStr">
+      <c r="B90" s="7" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C87" s="7" t="inlineStr">
+      <c r="C90" s="7" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="D87" s="7" t="inlineStr">
+      <c r="D90" s="7" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="E87" s="8" t="inlineStr">
+      <c r="E90" s="8" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="F87" s="8" t="inlineStr">
+      <c r="F90" s="8" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="G87" s="8" t="inlineStr">
+      <c r="G90" s="8" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="H87" s="8" t="inlineStr">
+      <c r="H90" s="8" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="I87" s="8" t="inlineStr"/>
-      <c r="J87" s="8" t="inlineStr">
+      <c r="I90" s="8" t="inlineStr"/>
+      <c r="J90" s="8" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="K87" s="8" t="inlineStr">
+      <c r="K90" s="8" t="inlineStr">
         <is>
           <t>⭐⭐⭐</t>
         </is>
       </c>
-      <c r="L87" s="8" t="inlineStr">
+      <c r="L90" s="8" t="inlineStr">
         <is>
           <t>⭐⭐⭐</t>
         </is>
       </c>
-      <c r="M87" s="8" t="inlineStr"/>
-      <c r="N87" s="8" t="inlineStr"/>
-      <c r="O87" s="8" t="inlineStr">
+      <c r="M90" s="8" t="inlineStr"/>
+      <c r="N90" s="8" t="inlineStr"/>
+      <c r="O90" s="8" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="P87" s="8" t="inlineStr"/>
-    </row>
-    <row r="88" ht="16" customHeight="1">
-      <c r="A88" s="10" t="inlineStr">
+      <c r="P90" s="8" t="inlineStr"/>
+    </row>
+    <row r="91" ht="16" customHeight="1">
+      <c r="A91" s="10" t="inlineStr">
         <is>
           <t>**PL-2: Cloud &amp; Cybersecurity Specialist**</t>
         </is>
       </c>
-      <c r="B88" s="9" t="inlineStr">
+      <c r="B91" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C88" s="9" t="inlineStr">
+      <c r="C91" s="9" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="D88" s="9" t="inlineStr">
+      <c r="D91" s="9" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="E88" s="10" t="inlineStr">
+      <c r="E91" s="10" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="F88" s="10" t="inlineStr">
+      <c r="F91" s="10" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="G88" s="10" t="inlineStr">
+      <c r="G91" s="10" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="H88" s="10" t="inlineStr"/>
-      <c r="I88" s="10" t="inlineStr">
+      <c r="H91" s="10" t="inlineStr"/>
+      <c r="I91" s="10" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="J88" s="10" t="inlineStr"/>
-      <c r="K88" s="10" t="inlineStr"/>
-      <c r="L88" s="10" t="inlineStr"/>
-      <c r="M88" s="10" t="inlineStr">
+      <c r="J91" s="10" t="inlineStr"/>
+      <c r="K91" s="10" t="inlineStr"/>
+      <c r="L91" s="10" t="inlineStr"/>
+      <c r="M91" s="10" t="inlineStr">
         <is>
           <t>⭐⭐⭐</t>
         </is>
       </c>
-      <c r="N88" s="10" t="inlineStr">
+      <c r="N91" s="10" t="inlineStr">
         <is>
           <t>⭐⭐⭐</t>
         </is>
       </c>
-      <c r="O88" s="10" t="inlineStr"/>
-      <c r="P88" s="10" t="inlineStr"/>
-    </row>
-    <row r="89" ht="16" customHeight="1">
-      <c r="A89" s="8" t="inlineStr">
+      <c r="O91" s="10" t="inlineStr"/>
+      <c r="P91" s="10" t="inlineStr"/>
+    </row>
+    <row r="92" ht="16" customHeight="1">
+      <c r="A92" s="8" t="inlineStr">
         <is>
           <t>**PL-3: UI/UX &amp; Digital Platform Engineer**</t>
         </is>
       </c>
-      <c r="B89" s="7" t="inlineStr">
+      <c r="B92" s="7" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C89" s="7" t="inlineStr">
+      <c r="C92" s="7" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="D89" s="7" t="inlineStr">
+      <c r="D92" s="7" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="E89" s="8" t="inlineStr">
+      <c r="E92" s="8" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="F89" s="8" t="inlineStr">
+      <c r="F92" s="8" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="G89" s="8" t="inlineStr"/>
-      <c r="H89" s="8" t="inlineStr">
+      <c r="G92" s="8" t="inlineStr"/>
+      <c r="H92" s="8" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="I89" s="8" t="inlineStr"/>
-      <c r="J89" s="8" t="inlineStr">
+      <c r="I92" s="8" t="inlineStr"/>
+      <c r="J92" s="8" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="K89" s="8" t="inlineStr"/>
-      <c r="L89" s="8" t="inlineStr"/>
-      <c r="M89" s="8" t="inlineStr"/>
-      <c r="N89" s="8" t="inlineStr"/>
-      <c r="O89" s="8" t="inlineStr">
+      <c r="K92" s="8" t="inlineStr"/>
+      <c r="L92" s="8" t="inlineStr"/>
+      <c r="M92" s="8" t="inlineStr"/>
+      <c r="N92" s="8" t="inlineStr"/>
+      <c r="O92" s="8" t="inlineStr">
         <is>
           <t>⭐⭐⭐</t>
         </is>
       </c>
-      <c r="P89" s="8" t="inlineStr">
+      <c r="P92" s="8" t="inlineStr">
         <is>
           <t>⭐⭐</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="16" customHeight="1">
-      <c r="A90" s="10" t="inlineStr">
+    <row r="93" ht="16" customHeight="1">
+      <c r="A93" s="10" t="inlineStr">
         <is>
           <t>**PL-4: IT Project Manager &amp; Technopreneur**</t>
         </is>
       </c>
-      <c r="B90" s="10" t="inlineStr">
+      <c r="B93" s="10" t="inlineStr">
         <is>
           <t>P3 / P1 / P2</t>
         </is>
       </c>
-      <c r="C90" s="9" t="inlineStr">
+      <c r="C93" s="9" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="D90" s="9" t="inlineStr">
+      <c r="D93" s="9" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="E90" s="10" t="inlineStr">
+      <c r="E93" s="10" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="F90" s="10" t="inlineStr">
+      <c r="F93" s="10" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="G90" s="10" t="inlineStr"/>
-      <c r="H90" s="10" t="inlineStr">
+      <c r="G93" s="10" t="inlineStr"/>
+      <c r="H93" s="10" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="I90" s="10" t="inlineStr">
+      <c r="I93" s="10" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="J90" s="10" t="inlineStr">
+      <c r="J93" s="10" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="K90" s="10" t="inlineStr">
+      <c r="K93" s="10" t="inlineStr">
         <is>
           <t>⭐</t>
         </is>
       </c>
-      <c r="L90" s="10" t="inlineStr"/>
-      <c r="M90" s="10" t="inlineStr"/>
-      <c r="N90" s="10" t="inlineStr"/>
-      <c r="O90" s="10" t="inlineStr">
+      <c r="L93" s="10" t="inlineStr"/>
+      <c r="M93" s="10" t="inlineStr"/>
+      <c r="N93" s="10" t="inlineStr"/>
+      <c r="O93" s="10" t="inlineStr">
         <is>
           <t>⭐⭐</t>
         </is>
       </c>
-      <c r="P90" s="10" t="inlineStr">
+      <c r="P93" s="10" t="inlineStr">
         <is>
           <t>⭐⭐⭐</t>
         </is>
       </c>
     </row>
-    <row r="91"/>
-    <row r="92" ht="20" customHeight="1">
-      <c r="A92" s="3" t="inlineStr">
+    <row r="94"/>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="3" t="inlineStr">
         <is>
           <t>7. MATRIKS PEMETAAN CPL ↔ 3 PROGRAM EDUCATIONAL OBJECTIVES (PEO)</t>
         </is>
       </c>
-      <c r="B92" s="4" t="n"/>
-      <c r="C92" s="4" t="n"/>
-      <c r="D92" s="4" t="n"/>
-      <c r="E92" s="4" t="n"/>
-      <c r="F92" s="5" t="n"/>
-    </row>
-    <row r="93" ht="26" customHeight="1">
-      <c r="A93" s="6" t="inlineStr">
+      <c r="B95" s="4" t="n"/>
+      <c r="C95" s="4" t="n"/>
+      <c r="D95" s="4" t="n"/>
+      <c r="E95" s="4" t="n"/>
+      <c r="F95" s="5" t="n"/>
+    </row>
+    <row r="96" ht="26" customHeight="1">
+      <c r="A96" s="6" t="inlineStr">
         <is>
           <t>Kode PEO</t>
         </is>
       </c>
-      <c r="B93" s="6" t="inlineStr">
+      <c r="B96" s="6" t="inlineStr">
         <is>
           <t>Nomenklatur Program Educational Objectives (3–5 Tahun)</t>
         </is>
       </c>
-      <c r="C93" s="6" t="inlineStr">
+      <c r="C96" s="6" t="inlineStr">
         <is>
           <t>CPL Sikap &amp; Umum</t>
         </is>
       </c>
-      <c r="D93" s="6" t="inlineStr">
+      <c r="D96" s="6" t="inlineStr">
         <is>
           <t>CPL Pengetahuan</t>
         </is>
       </c>
-      <c r="E93" s="6" t="inlineStr">
+      <c r="E96" s="6" t="inlineStr">
         <is>
           <t>CPL Keterampilan Khusus</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="16" customHeight="1">
-      <c r="A94" s="8" t="inlineStr">
+    <row r="97" ht="16" customHeight="1">
+      <c r="A97" s="8" t="inlineStr">
         <is>
           <t>**PEO-1**</t>
         </is>
       </c>
-      <c r="B94" s="8" t="inlineStr">
+      <c r="B97" s="8" t="inlineStr">
         <is>
           <t>**PEO-1 — Professional Practice and Systems Integration**&lt;br/&gt;Lulusan menunjukkan keunggulan profesional dalam merancang, mengintegrasikan, dan mengelola sistem informasi cerdas, infrastruktur cloud, atau platform digital enterprise.</t>
         </is>
       </c>
-      <c r="C94" s="8" t="inlineStr">
+      <c r="C97" s="8" t="inlineStr">
         <is>
           <t>`S1`, `KU1`, `KU2`, `KU3`</t>
         </is>
       </c>
-      <c r="D94" s="8" t="inlineStr">
+      <c r="D97" s="8" t="inlineStr">
         <is>
           <t>`P1`, `P2`, `P3`, `P4`</t>
         </is>
       </c>
-      <c r="E94" s="8" t="inlineStr">
+      <c r="E97" s="8" t="inlineStr">
         <is>
           <t>`KK1`, `KK2`, `KK3`, `KK4`, `KK5`</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="16" customHeight="1">
-      <c r="A95" s="10" t="inlineStr">
+    <row r="98" ht="16" customHeight="1">
+      <c r="A98" s="10" t="inlineStr">
         <is>
           <t>**PEO-2**</t>
         </is>
       </c>
-      <c r="B95" s="10" t="inlineStr">
+      <c r="B98" s="10" t="inlineStr">
         <is>
           <t>**PEO-2 — Digital Innovation and Technopreneurship**&lt;br/&gt;Lulusan mampu memimpin inovasi digital, menginisiasi usaha rintisan teknologi (*technopreneurship*), atau mengelola proyek transformasi digital yang memberikan dampak ekonomi dan sosial.</t>
         </is>
       </c>
-      <c r="C95" s="10" t="inlineStr">
+      <c r="C98" s="10" t="inlineStr">
         <is>
           <t>`S1`, `KU1`, `KU2`, `KU3`</t>
         </is>
       </c>
-      <c r="D95" s="10" t="inlineStr">
+      <c r="D98" s="10" t="inlineStr">
         <is>
           <t>`P2`, `P3`, `P4`</t>
         </is>
       </c>
-      <c r="E95" s="10" t="inlineStr">
+      <c r="E98" s="10" t="inlineStr">
         <is>
           <t>`KK6`, `KK5`, `KK1`</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="16" customHeight="1">
-      <c r="A96" s="8" t="inlineStr">
+    <row r="99" ht="16" customHeight="1">
+      <c r="A99" s="8" t="inlineStr">
         <is>
           <t>**PEO-3**</t>
         </is>
       </c>
-      <c r="B96" s="8" t="inlineStr">
+      <c r="B99" s="8" t="inlineStr">
         <is>
           <t>**PEO-3 — Advanced Study, Research, and Lifelong Learning**&lt;br/&gt;Lulusan mampu melanjutkan studi ke jenjang pascasarjana, melakukan riset terapan di bidang sains komputasi/AI, serta adaptif mengembangkan diri sepanjang hayat.</t>
         </is>
       </c>
-      <c r="C96" s="8" t="inlineStr">
+      <c r="C99" s="8" t="inlineStr">
         <is>
           <t>`S1`, `KU1`, `KU2`, `KU3`</t>
         </is>
       </c>
-      <c r="D96" s="8" t="inlineStr">
+      <c r="D99" s="8" t="inlineStr">
         <is>
           <t>`P1`, `P2`, `P3`, `P4`</t>
         </is>
       </c>
-      <c r="E96" s="8" t="inlineStr">
+      <c r="E99" s="8" t="inlineStr">
         <is>
           <t>`KK1`, `KK2`, `KK3`, `KK4`, `KK5`, `KK6`</t>
         </is>
@@ -3277,16 +3403,16 @@
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A85:P85"/>
-    <mergeCell ref="A92:F92"/>
     <mergeCell ref="A46:P46"/>
     <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A88:P88"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A70:P70"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A20:F20"/>
     <mergeCell ref="A29:F29"/>
     <mergeCell ref="A7:F7"/>
-    <mergeCell ref="A68:P68"/>
+    <mergeCell ref="A95:F95"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>